<commit_message>
remove duplication device id A2027
</commit_message>
<xml_diff>
--- a/1.training_model/dummy_data/UGS_A2027.xlsx
+++ b/1.training_model/dummy_data/UGS_A2027.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\Documents\Device_Identifier\Dummy data\Structured_df\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sitisyaziyah\source\repos\DeviceCluster\1.training_model\dummy_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CC5740C2-B712-44A4-9B24-847BFE2CB7DC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E612624-0F62-4CEF-A592-759555FA1E4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{4A364C8F-793E-478C-AA2B-3EB646C3E912}"/>
   </bookViews>
@@ -7053,7 +7053,7 @@
         <v>281</v>
       </c>
       <c r="D329" t="s">
-        <v>139</v>
+        <v>89</v>
       </c>
       <c r="E329" t="s">
         <v>330</v>

</xml_diff>